<commit_message>
Reaggregate data with latest processing reports (3,649 records)
Added __future__ annotations import for Python 3.9 compatibility.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/aggregated_notes.xlsx
+++ b/data/aggregated_notes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2353,6 +2353,302 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>late start maintenance</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AUTO TIE BALER</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Darius</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>LD was supersack w/loose LD bales</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Jay</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Tony left early, Jay had to sort pallets, cut pallets, and load on the belt</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>downtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Clarence</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>finished HD - opened up shredder and granulator and cleaned them out - switched to LD purge</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Darius, Clarnce</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>machine was overheating</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Clarence</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>single shaft thermal cut off alarm kept appearing - had to reset machine before blowing a fuse</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Clarence</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>started at 1030 - it went down on second shift yesterday - got it going for a couple of hours and another fuse blew</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>downtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>had to do a blade change - hand feeing the grinder waiting on maintenance to finish the shredder</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add week of 3/30/26-4/3/26 data and rebuild dashboards
- 3 new shift reports (1st, 2nd, 3rd) for week of 3/30/26-4/3/26
- Re-aggregated: 3784 → 3841 records (+57 new rows)
- Rebuilt weekly, daily, and operator dashboards

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/aggregated_notes.xlsx
+++ b/data/aggregated_notes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2649,6 +2649,80 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>no weights entered - late start, had to wait for material</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Clarence</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>the first 3.5 hours were spent jumping in and out of the machine - the modifications were made for regular sized plastic pallets - the pallets that were run were a lot longer</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add week of 4/6/26-4/10/26 data, profit dashboard, and rebuild all dashboards
- Added 63 new records (3841 → 3904 total) from week of 4/6-4/10
- Added profit margin simulator dashboard (src/build_profit_dashboard.py)
- Rebuilt interactive, daily, operator, and profit dashboards

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/aggregated_notes.xlsx
+++ b/data/aggregated_notes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2723,6 +2723,154 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Clarence</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Clarence had to keep jumping in and out of machine</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>belt under shredder stopped working</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>downtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Clarence</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>came in and the belt for the shredder was not working - switching material - Chad is going to help with new material</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>downtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>GRINDER</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Clarence</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>switching from HDPE to HIPS</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add week of 4/20/26-4/24/26 data via Gmail API fetcher
First end-to-end run of the new src/fetch_emails.py Gmail API fetcher:
- Auto-detected new processing-weights email and downloaded 3 shift xlsx files
- Auto-renamed using the date range parsed from the email subject
- Idempotent skip on payroll PDFs already present (5 detected, 0 downloaded)

Pipeline:
  fetch_emails.py --all → aggregate_daily_data.py → build_*_dashboard.py

- 67 new daily records (3970 → 4037 total)
- 1 duplicate dropped during aggregation
- Payroll uplift refined to +14.5% (2012h gap / 13839h production)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/aggregated_notes.xlsx
+++ b/data/aggregated_notes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>